<commit_message>
Register command-set code OT (OTH-AT) in the code register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/M2M_Code Register.xlsx
+++ b/doc/M2M_Code Register.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\doc\1.Projects\ESP\표준모델\03_설계문서\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Doc\1.Projects\ESP\표준모델\03_설계문서\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE4C70E-1717-4B7C-97EB-7B51E9F1F091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A2ACFC-5DEE-4E6F-8FF1-D2B4305D26E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6540" yWindow="960" windowWidth="32475" windowHeight="18885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="315" yWindow="1245" windowWidth="32475" windowHeight="18885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="보드코드" sheetId="1" r:id="rId1"/>
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="219">
   <si>
     <t>M2M 보드 코드 할당 대장 (BOARD, 3자리 = 구분 1자 + 일련 1자 + 리비전 1자)</t>
   </si>
@@ -748,6 +748,30 @@
   </si>
   <si>
     <t>AT UART / Log UART 핀 열 삭제 — 보드 핀맵은 보드별 빌드 설정(CONFIG)에서 확인</t>
+  </si>
+  <si>
+    <t>OT</t>
+  </si>
+  <si>
+    <t>OTH-AT 호환 (OTH Platform)</t>
+  </si>
+  <si>
+    <t>AT*OTH*&lt;명령&gt;</t>
+  </si>
+  <si>
+    <t>OTH-AT Compatible Command Set - *.docx</t>
+  </si>
+  <si>
+    <t>OTH 빌드(Kconfig AT_MODEM_CMDSET_OTH)에서 자동 선택. 이미지 ID ..._OT_&lt;고객&gt;&lt;REL&gt; (M2M 이미지와 OTA/FOTA 상호 거부)</t>
+  </si>
+  <si>
+    <t>명령체계코드</t>
+  </si>
+  <si>
+    <t>OTH-AT 호환 명령 체계 신규 등록 (OTH_ESP32_C3 빌드, M2M_CMD_CODE 자동 선택)</t>
+  </si>
+  <si>
+    <t>2026-10-06</t>
   </si>
 </sst>
 </file>
@@ -868,7 +892,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -909,6 +933,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1322,29 +1349,29 @@
       </c>
     </row>
     <row r="2" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="17"/>
-      <c r="S2" s="17"/>
-      <c r="T2" s="17"/>
-      <c r="U2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
+      <c r="U2" s="18"/>
     </row>
     <row r="4" spans="1:21" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -1671,7 +1698,7 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -9991,7 +10018,7 @@
     </row>
     <row r="197" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A197" s="3" t="str">
-        <f t="shared" ref="A197:A228" si="18">IF(B197="","",ROW()-4)</f>
+        <f t="shared" ref="A197:A200" si="18">IF(B197="","",ROW()-4)</f>
         <v/>
       </c>
       <c r="B197" s="11"/>
@@ -10021,7 +10048,7 @@
         <v/>
       </c>
       <c r="S197" s="5" t="str">
-        <f t="shared" ref="S197:S228" si="19">IF(R197="","","M2M_"&amp;R197&amp;"_AT-MM-"&amp;IF(M197="","UART",M197)&amp;"_V01.00_"&amp;IF(N197="","AC0",N197)&amp;"_0FN_YYMMDD.zip")</f>
+        <f t="shared" ref="S197:S200" si="19">IF(R197="","","M2M_"&amp;R197&amp;"_AT-MM-"&amp;IF(M197="","UART",M197)&amp;"_V01.00_"&amp;IF(N197="","AC0",N197)&amp;"_0FN_YYMMDD.zip")</f>
         <v/>
       </c>
       <c r="T197" s="3" t="str">
@@ -10574,14 +10601,14 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="4" spans="1:6" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -11112,18 +11139,18 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
     </row>
     <row r="4" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -12295,17 +12322,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="4" spans="1:9" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -12454,18 +12481,34 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
+    <row r="9" spans="1:9" ht="51" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>215</v>
+      </c>
       <c r="I9" s="3" t="str">
         <f>IF(A9="","",IF(LEN(A9)&lt;&gt;2,"2자리 아님",IF(SUMPRODUCT(--ISERROR(FIND(MID(A9,{1,2},1),"ABCDEFGHIJKLMNOPQRSTUVWXYZ")))&gt;0,"문자 오류",IF(COUNTIF($A$5:$A$40,A9)&gt;1,"중복","OK"))))</f>
-        <v/>
+        <v>OK</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -12952,16 +12995,16 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
     </row>
     <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -16100,7 +16143,7 @@
     <row r="197" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A197" s="11"/>
       <c r="B197" s="3" t="str">
-        <f t="shared" ref="B197:B228" si="6">IF(A197="","",IF(LEFT(A197,1)="A","내부",IF(LEFT(A197,1)="Z","예비","고객사")))</f>
+        <f t="shared" ref="B197:B200" si="6">IF(A197="","",IF(LEFT(A197,1)="A","내부",IF(LEFT(A197,1)="Z","예비","고객사")))</f>
         <v/>
       </c>
       <c r="C197" s="12"/>
@@ -16193,7 +16236,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -16249,6 +16292,21 @@
       </c>
       <c r="E3" s="6"/>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="E4" s="6"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>